<commit_message>
v1.2.0 XSSF 모드 폐지, merge/bundle/이미지 URL 기능 추가, 문서 갱신
- XSSF(비스트리밍) 모드 폐지, 항상 스트리밍 모드로 동작
- 자동 셀 병합(merge), 요소 묶음(bundle), 이미지 URL 지원 추가
- RIGHT repeat 열 너비 복제/간접 겹침 검사 버그 수정
- 문서 갱신: 신규 기능 반영, 의존성 예제 보강
</commit_message>
<xml_diff>
--- a/modules/tbeg/src/test/resources/templates/rich_sample_template.xlsx
+++ b/modules/tbeg/src/test/resources/templates/rich_sample_template.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hyh/dev/mylib/kotlin/kotlin-common-library/modules/report/template-based-excel-generator/src/test/resources/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0C75FF3-9173-C848-A13D-DD0436089829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DF67C16-0F1F-5244-977D-7B0E9821CA88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="68740" yWindow="1000" windowWidth="25540" windowHeight="23100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="69780" yWindow="280" windowWidth="27580" windowHeight="23100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sales Report" sheetId="1" r:id="rId1"/>
+    <sheet name="Sales Report (Right)" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="41">
   <si>
     <t>${reportTitle}</t>
   </si>
@@ -47,6 +48,12 @@
     <t>Date: ${reportDate}</t>
   </si>
   <si>
+    <t>${repeat(depts, B8:G8, d)}</t>
+  </si>
+  <si>
+    <t>${repeat(products, I8:K8, p)}</t>
+  </si>
+  <si>
     <t>Department</t>
   </si>
   <si>
@@ -95,19 +102,62 @@
     <t>Average</t>
   </si>
   <si>
+    <t>${repeat(employees, B31:K31, emp)}</t>
+  </si>
+  <si>
+    <t>${bundle(range=B30:K33)}</t>
+  </si>
+  <si>
+    <t>${subtitle_emp}</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Rank</t>
+  </si>
+  <si>
+    <t>${merge(emp.dept)}</t>
+  </si>
+  <si>
+    <t>${merge(emp.team)}</t>
+  </si>
+  <si>
+    <t>${emp.name}</t>
+  </si>
+  <si>
+    <t>${emp.rank}</t>
+  </si>
+  <si>
+    <t>${emp.revenue}</t>
+  </si>
+  <si>
+    <t>${emp.cost}</t>
+  </si>
+  <si>
+    <t>${emp.target}</t>
+  </si>
+  <si>
+    <t>${image(logo,,-1:0)}</t>
+  </si>
+  <si>
     <t>${image(ci)}</t>
   </si>
   <si>
-    <t>${image(logo,,-1:0)}</t>
-    <phoneticPr fontId="14" type="noConversion"/>
-  </si>
-  <si>
-    <t>${repeat(depts, B8:G8, d)}</t>
-    <phoneticPr fontId="14" type="noConversion"/>
-  </si>
-  <si>
-    <t>${repeat(products, I8:K8, p)}</t>
-    <phoneticPr fontId="14" type="noConversion"/>
+    <t>${repeat(collection=depts, range=C8:C13, var=d, direction=RIGHT)}</t>
+  </si>
+  <si>
+    <t>${repeat(collection=employees, range=H8:H16, var=emp, direction=RIGHT)}</t>
+  </si>
+  <si>
+    <t>${bundle(range=G7:J16)}</t>
+  </si>
+  <si>
+    <t>${repeat(collection=products, range=C15:C17, var=p, direction=RIGHT)}</t>
+    <phoneticPr fontId="8" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -121,12 +171,6 @@
       <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="55"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -171,36 +215,6 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="8"/>
       <name val="맑은 고딕"/>
       <family val="3"/>
@@ -234,8 +248,54 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <u/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <u/>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -258,8 +318,38 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2F5496"/>
+        <bgColor rgb="FF2F5496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F3864"/>
+        <bgColor rgb="FF1F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1B5E5E"/>
+        <bgColor rgb="FF1B5E5E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E2F3"/>
+        <bgColor rgb="FFD9E2F3"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="19">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -507,114 +597,473 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="11" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="13" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="11" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="13" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="13" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="13" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="3" fontId="16" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="16" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="16" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="16" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="16" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="12">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color indexed="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor indexed="45"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color indexed="17"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor indexed="42"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color indexed="10"/>
@@ -707,6 +1156,11 @@
           <c:tx>
             <c:v>Revenue</c:v>
           </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
           <c:invertIfNegative val="1"/>
           <c:cat>
             <c:strRef>
@@ -733,7 +1187,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-EC55-F74B-B3AA-9FCBDD2D5CE5}"/>
+              <c16:uniqueId val="{00000000-DC83-F74F-AAF4-B258015A5F5A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -743,6 +1197,11 @@
           <c:tx>
             <c:v>Cost</c:v>
           </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
           <c:invertIfNegative val="1"/>
           <c:cat>
             <c:strRef>
@@ -769,7 +1228,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-EC55-F74B-B3AA-9FCBDD2D5CE5}"/>
+              <c16:uniqueId val="{00000001-DC83-F74F-AAF4-B258015A5F5A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -779,6 +1238,11 @@
           <c:tx>
             <c:v>Profit</c:v>
           </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
           <c:invertIfNegative val="1"/>
           <c:cat>
             <c:strRef>
@@ -805,7 +1269,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-EC55-F74B-B3AA-9FCBDD2D5CE5}"/>
+              <c16:uniqueId val="{00000002-DC83-F74F-AAF4-B258015A5F5A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -908,6 +1372,11 @@
           <c:tx>
             <c:v>Revenue</c:v>
           </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
           <c:cat>
             <c:strRef>
               <c:f>'Sales Report'!$I$8</c:f>
@@ -933,7 +1402,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-C1BE-F146-A5E7-9922092E064B}"/>
+              <c16:uniqueId val="{00000000-A6A9-6641-B037-5346D2BF445D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -982,7 +1451,7 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Diagramm0">
+        <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
@@ -1018,7 +1487,7 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Diagramm1">
+        <xdr:cNvPr id="3" name="Chart 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
@@ -1362,214 +1831,697 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K29"/>
+  <dimension ref="B2:K36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="3" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="11" width="14" customWidth="1"/>
+    <col min="2" max="2" width="18" style="44" customWidth="1"/>
+    <col min="3" max="7" width="14" style="44" customWidth="1"/>
+    <col min="8" max="8" width="3" style="44" customWidth="1"/>
+    <col min="9" max="9" width="18" style="44" customWidth="1"/>
+    <col min="10" max="11" width="14" style="44" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="50" customHeight="1">
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="29"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
+      <c r="I2" s="51"/>
+      <c r="J2" s="51"/>
+      <c r="K2" s="51"/>
     </row>
     <row r="3" spans="2:11" ht="30" customHeight="1">
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
-      <c r="K3" s="29"/>
+      <c r="B3" s="51"/>
+      <c r="C3" s="51"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="51"/>
+      <c r="G3" s="51"/>
+      <c r="H3" s="51"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="51"/>
+      <c r="K3" s="51"/>
     </row>
     <row r="4" spans="2:11" ht="22" customHeight="1">
       <c r="C4" s="1"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="27" t="s">
+      <c r="F4" s="13" t="s">
         <v>1</v>
       </c>
       <c r="G4" s="1"/>
-      <c r="I4" s="32" t="s">
+      <c r="I4" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="J4" s="33"/>
-      <c r="K4" s="32" t="s">
+      <c r="J4" s="17"/>
+      <c r="K4" s="16" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="2:11" ht="8" customHeight="1"/>
     <row r="6" spans="2:11" ht="18" customHeight="1" thickBot="1">
-      <c r="B6" s="26" t="s">
-        <v>22</v>
-      </c>
-      <c r="I6" s="26" t="s">
-        <v>23</v>
+      <c r="B6" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="I6" s="12" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="2:11" ht="28" customHeight="1">
-      <c r="B7" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D7" s="7" t="s">
+      <c r="B7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="C7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="D7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="E7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I7" s="14" t="s">
+      <c r="F7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J7" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="K7" s="16" t="s">
+      <c r="G7" s="5" t="s">
         <v>11</v>
       </c>
+      <c r="I7" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="8" spans="2:11" ht="24" customHeight="1" thickBot="1">
-      <c r="B8" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="B8" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="4" t="e">
+      <c r="C8" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="2" t="e">
         <f>C8-D8</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" s="9" t="e">
+      <c r="F8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="6" t="e">
         <f>C8/F8</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I8" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="J8" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="K8" s="9" t="e">
+      <c r="I8" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="K8" s="6" t="e">
         <f>J8/J9</f>
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="9" spans="2:11" ht="24" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B9" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="19">
+      <c r="B9" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="24">
         <f>SUM(C8:C8)</f>
         <v>0</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="25">
         <f>SUM(D8:D8)</f>
         <v>0</v>
       </c>
-      <c r="E9" s="5" t="e">
+      <c r="E9" s="25" t="e">
         <f>SUM(E8:E8)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="25">
         <f>SUM(F8:F8)</f>
         <v>0</v>
       </c>
-      <c r="G9" s="10" t="e">
+      <c r="G9" s="26" t="e">
         <f>C9/F9</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="I9" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="J9" s="24">
+      <c r="I9" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="J9" s="33">
         <f>SUM(J8:J8)</f>
         <v>0</v>
       </c>
-      <c r="K9" s="17">
+      <c r="K9" s="34">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="2:11" ht="24" customHeight="1" thickBot="1">
-      <c r="B10" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="20" t="e">
+      <c r="B10" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="28" t="e">
         <f>AVERAGE(C8:C8)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D10" s="11" t="e">
+      <c r="D10" s="29" t="e">
         <f>AVERAGE(D8:D8)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E10" s="11" t="e">
+      <c r="E10" s="29" t="e">
         <f>AVERAGE(E8:E8)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F10" s="12"/>
-      <c r="G10" s="13"/>
-    </row>
-    <row r="29" spans="6:11" ht="18" customHeight="1">
-      <c r="F29" s="2"/>
-      <c r="G29" s="3"/>
-      <c r="J29" s="30" t="s">
+      <c r="F10" s="30"/>
+      <c r="G10" s="31"/>
+    </row>
+    <row r="28" spans="2:11">
+      <c r="B28" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D28" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="29" spans="2:11" ht="29" customHeight="1" thickBot="1">
+      <c r="D29" s="48" t="s">
+        <v>24</v>
+      </c>
+      <c r="E29" s="49"/>
+      <c r="F29" s="49"/>
+      <c r="G29" s="49"/>
+      <c r="H29" s="49"/>
+      <c r="I29" s="49"/>
+      <c r="J29" s="14"/>
+      <c r="K29" s="15"/>
+    </row>
+    <row r="30" spans="2:11">
+      <c r="B30" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="H30" s="4"/>
+      <c r="I30" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="J30" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K30" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="31" spans="2:11">
+      <c r="B31" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C31" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="D31" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="E31" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="F31" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="G31" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="I31" s="18" t="e">
+        <f>F31-G31</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="J31" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="K31" s="22" t="e">
+        <f>F31/J31</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="32" spans="2:11">
+      <c r="B32" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="C32" s="36"/>
+      <c r="D32" s="36"/>
+      <c r="E32" s="36"/>
+      <c r="F32" s="36">
+        <f>SUM(F31:F31)</f>
+        <v>0</v>
+      </c>
+      <c r="G32" s="36">
+        <f>SUM(G31:G31)</f>
+        <v>0</v>
+      </c>
+      <c r="H32" s="37"/>
+      <c r="I32" s="38" t="e">
+        <f>SUM(I31:I31)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="J32" s="36">
+        <f>SUM(J31:J31)</f>
+        <v>0</v>
+      </c>
+      <c r="K32" s="39" t="e">
+        <f>F32/J32</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="33" spans="2:11" ht="18" customHeight="1" thickBot="1">
+      <c r="B33" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="K29" s="31" t="s">
-        <v>20</v>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41" t="e">
+        <f>AVERAGE(F31:F31)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G33" s="41" t="e">
+        <f>AVERAGE(G31:G31)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H33" s="42"/>
+      <c r="I33" s="41" t="e">
+        <f>AVERAGE(I31:I31)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="J33" s="42"/>
+      <c r="K33" s="43"/>
+    </row>
+    <row r="36" spans="2:11">
+      <c r="J36" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="K36" s="15" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="D29:I29"/>
     <mergeCell ref="B2:K3"/>
   </mergeCells>
-  <phoneticPr fontId="14" type="noConversion"/>
+  <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="G8">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="11" priority="5" operator="greaterThanOrEqual">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="10" priority="6" operator="lessThan">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K8">
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="9" priority="7" operator="greaterThanOrEqual">
       <formula>0.3</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="8" operator="lessThan">
       <formula>0.3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K31">
+    <cfRule type="cellIs" dxfId="7" priority="1" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="2" stopIfTrue="1" operator="lessThan">
+      <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A2:K19"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
+  <cols>
+    <col min="1" max="1" width="3" style="44" customWidth="1"/>
+    <col min="2" max="2" width="18" style="44" customWidth="1"/>
+    <col min="3" max="5" width="14" style="44" customWidth="1"/>
+    <col min="6" max="6" width="16.5" style="44" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18" style="44" customWidth="1"/>
+    <col min="8" max="10" width="14" style="44" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:11" ht="50" customHeight="1">
+      <c r="B2" s="53" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
+      <c r="I2" s="51"/>
+      <c r="J2" s="51"/>
+      <c r="K2" s="54"/>
+    </row>
+    <row r="3" spans="2:11" ht="30" customHeight="1">
+      <c r="B3" s="51"/>
+      <c r="C3" s="51"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="51"/>
+      <c r="G3" s="51"/>
+      <c r="H3" s="51"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="51"/>
+      <c r="K3" s="54"/>
+    </row>
+    <row r="4" spans="2:11" ht="22" customHeight="1">
+      <c r="B4" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="F4" t="s">
+        <v>2</v>
+      </c>
+      <c r="I4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" ht="8" customHeight="1"/>
+    <row r="6" spans="2:11" ht="18" customHeight="1">
+      <c r="B6" s="46" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" s="46" t="s">
+        <v>38</v>
+      </c>
+      <c r="I6" s="46" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" ht="29" customHeight="1" thickBot="1">
+      <c r="G7" s="52" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="51"/>
+    </row>
+    <row r="8" spans="2:11" ht="24" customHeight="1">
+      <c r="B8" s="63" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="56" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="69" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="57" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" s="63" t="s">
+        <v>6</v>
+      </c>
+      <c r="H8" s="56" t="s">
+        <v>28</v>
+      </c>
+      <c r="I8" s="69" t="s">
+        <v>20</v>
+      </c>
+      <c r="J8" s="57" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" ht="24" customHeight="1">
+      <c r="B9" s="64" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="59" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="70">
+        <f>SUM(C9:C9)</f>
+        <v>0</v>
+      </c>
+      <c r="E9" s="60" t="e">
+        <f>AVERAGE(C9:C9)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G9" s="64" t="s">
+        <v>25</v>
+      </c>
+      <c r="H9" s="68" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" s="72"/>
+      <c r="J9" s="65"/>
+    </row>
+    <row r="10" spans="2:11" ht="24" customHeight="1">
+      <c r="B10" s="64" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="59" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="70">
+        <f>SUM(C10:C10)</f>
+        <v>0</v>
+      </c>
+      <c r="E10" s="60" t="e">
+        <f>AVERAGE(C10:C10)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G10" s="64" t="s">
+        <v>26</v>
+      </c>
+      <c r="H10" s="68" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" s="72"/>
+      <c r="J10" s="65"/>
+    </row>
+    <row r="11" spans="2:11" ht="24" customHeight="1">
+      <c r="B11" s="64" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="59" t="e">
+        <f>C9-C10</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D11" s="70" t="e">
+        <f>SUM(C11:C11)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E11" s="60" t="e">
+        <f>AVERAGE(C11:C11)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="G11" s="64" t="s">
+        <v>27</v>
+      </c>
+      <c r="H11" s="68" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11" s="72"/>
+      <c r="J11" s="65"/>
+    </row>
+    <row r="12" spans="2:11" ht="24" customHeight="1">
+      <c r="B12" s="64" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="59" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" s="70">
+        <f>SUM(C12:C12)</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="65"/>
+      <c r="G12" s="64" t="s">
+        <v>7</v>
+      </c>
+      <c r="H12" s="59" t="s">
+        <v>32</v>
+      </c>
+      <c r="I12" s="70">
+        <f>SUM(H12:H12)</f>
+        <v>0</v>
+      </c>
+      <c r="J12" s="60" t="e">
+        <f>AVERAGE(H12:H12)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" ht="24" customHeight="1" thickBot="1">
+      <c r="B13" s="66" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="62" t="e">
+        <f>C9/C12</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D13" s="71" t="e">
+        <f>D9/D12</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E13" s="67"/>
+      <c r="G13" s="64" t="s">
+        <v>8</v>
+      </c>
+      <c r="H13" s="59" t="s">
+        <v>33</v>
+      </c>
+      <c r="I13" s="70">
+        <f>SUM(H13:H13)</f>
+        <v>0</v>
+      </c>
+      <c r="J13" s="60" t="e">
+        <f>AVERAGE(H13:H13)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" ht="24" customHeight="1" thickBot="1">
+      <c r="B14" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="G14" s="64" t="s">
+        <v>9</v>
+      </c>
+      <c r="H14" s="59" t="e">
+        <f>H12-H13</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I14" s="70" t="e">
+        <f>SUM(H14:H14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="J14" s="60" t="e">
+        <f>AVERAGE(H14:H14)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="15" spans="2:11" ht="24" customHeight="1">
+      <c r="B15" s="55" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="56" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="73" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" s="64" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" s="59" t="s">
+        <v>34</v>
+      </c>
+      <c r="I15" s="70">
+        <f>SUM(H15:H15)</f>
+        <v>0</v>
+      </c>
+      <c r="J15" s="65"/>
+    </row>
+    <row r="16" spans="2:11" ht="24" customHeight="1" thickBot="1">
+      <c r="B16" s="58" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="59" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" s="74">
+        <f>SUM(C16:C16)</f>
+        <v>0</v>
+      </c>
+      <c r="G16" s="66" t="s">
+        <v>11</v>
+      </c>
+      <c r="H16" s="62" t="e">
+        <f>H12/H15</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I16" s="71" t="e">
+        <f>I12/I15</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J16" s="67"/>
+    </row>
+    <row r="17" spans="2:11" ht="24" customHeight="1" thickBot="1">
+      <c r="B17" s="61" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" s="62" t="e">
+        <f>C16/D16</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D17" s="75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" ht="18" customHeight="1">
+      <c r="J18" s="47" t="s">
+        <v>35</v>
+      </c>
+      <c r="K18" s="46" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" ht="24" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="B2:K3"/>
+  </mergeCells>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <conditionalFormatting sqref="C13">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThanOrEqual">
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C17">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThanOrEqual">
+      <formula>0.3</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="4" operator="lessThan">
+      <formula>0.3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H16">
+    <cfRule type="cellIs" dxfId="1" priority="5" operator="greaterThanOrEqual">
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="6" operator="lessThan">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>